<commit_message>
chore(ground-truth): batch-link XLSX to video_jobs + spawn 5 new workbooks
Existing GT workbooks weren't linked to video_jobs by video_job_id, so
eval-match.js couldn't cleanly pair truth files with pipeline runs.
Patches all linkable XLSX by keeper+date+opponent match and rebuilds
their JSONs — 15 of 16 workbooks now cleanly linked.

Spawns fresh workbooks for Amalie's BC Soccer match (2026-02-27 vs CMF 2008)
+ 4 untagged Judah matches from June, video_job_id pre-filled so
eval-match.js runs immediately after tagging.

Also adds:
- ground-truth-coverage: audit of GT-to-video_job coverage per keeper
- link-ground-truth-to-jobs: the batch patcher itself (idempotent)
- fix-amalie-match-date: corrects VEO's 2026-02-27 (form had 2026-02-08)
- peek-video-job, diagnose-amalie-job: one-off diagnostics for stuck runs

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/ground-truth/judah-2026-06-14-kcity-2016-gold.xlsx
+++ b/scripts/ground-truth/judah-2026-06-14-kcity-2016-gold.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="98">
   <si>
     <t>STIX Match Ground-Truth Tagger</t>
   </si>
@@ -174,6 +174,9 @@
   </si>
   <si>
     <t>video_job_id</t>
+  </si>
+  <si>
+    <t>83b3a438-99fa-4463-9e1b-41bcab523104</t>
   </si>
   <si>
     <t>Fill in after upload — needed for eval</t>
@@ -1037,10 +1040,10 @@
         <v>51</v>
       </c>
       <c r="B14" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1080,34 +1083,34 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>30</v>
@@ -1789,43 +1792,43 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>62</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>30</v>
@@ -2525,7 +2528,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -2535,7 +2538,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -2545,7 +2548,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
@@ -2553,7 +2556,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
         <v>1</v>
@@ -2561,7 +2564,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -2569,7 +2572,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B7" t="s">
         <v>1</v>
@@ -2577,7 +2580,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
         <v>1</v>
@@ -2585,7 +2588,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B9" t="s">
         <v>1</v>
@@ -2593,7 +2596,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
@@ -2601,7 +2604,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B11" t="s">
         <v>1</v>
@@ -2609,7 +2612,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B12" t="s">
         <v>1</v>
@@ -2617,7 +2620,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
@@ -2625,34 +2628,34 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K16" s="4" t="s">
         <v>30</v>
@@ -3340,28 +3343,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>30</v>
@@ -4040,25 +4043,25 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>30</v>
@@ -4728,16 +4731,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>30</v>

</xml_diff>